<commit_message>
chore(import): items 2-5 re-imported (85 pages + onboard-delights again), uploaded and previewed; spot-checks, fixes.json entries, report rows
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-app-entry.report.xlsx
+++ b/tools/importer/reports/import-app-entry.report.xlsx
@@ -1030,7 +1030,7 @@
     <t>app-entry</t>
   </si>
   <si>
-    <t>2026-10-24T00:55:47.134Z</t>
+    <t>2026-10-24T08:28:12.608Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/flugsuche</t>
@@ -1162,7 +1162,7 @@
     <t>at/de/gepaeck</t>
   </si>
   <si>
-    <t>2026-10-24T00:57:44.935Z</t>
+    <t>2026-10-24T08:19:23.748Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/gepaeck</t>
@@ -1735,7 +1735,7 @@
     <t>at/de/miles-and-more</t>
   </si>
   <si>
-    <t>2026-10-24T00:57:52.050Z</t>
+    <t>2026-10-24T08:19:25.609Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/miles-and-more</t>
@@ -3448,7 +3448,7 @@
     <t>de/de/flugsuche</t>
   </si>
   <si>
-    <t>2026-10-24T00:55:57.428Z</t>
+    <t>2026-10-24T08:28:14.965Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/flugsuche</t>
@@ -3559,7 +3559,7 @@
     <t>de/de/gepaeck</t>
   </si>
   <si>
-    <t>2026-10-24T00:58:07.054Z</t>
+    <t>2026-10-24T08:19:28.205Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/gepaeck</t>
@@ -4075,7 +4075,7 @@
     <t>de/de/miles-and-more</t>
   </si>
   <si>
-    <t>2026-10-24T00:58:13.904Z</t>
+    <t>2026-10-24T08:19:30.412Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/miles-and-more</t>
@@ -5161,7 +5161,7 @@
     <t>de/en/baggage</t>
   </si>
   <si>
-    <t>2026-10-24T00:58:30.914Z</t>
+    <t>2026-10-24T08:19:33.950Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/baggage</t>
@@ -5761,7 +5761,7 @@
     <t>de/en/flight-search</t>
   </si>
   <si>
-    <t>2026-10-24T00:56:05.999Z</t>
+    <t>2026-10-24T08:28:17.338Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/flight-search</t>
@@ -6322,7 +6322,7 @@
     <t>de/en/miles-and-more</t>
   </si>
   <si>
-    <t>2026-10-24T00:58:43.146Z</t>
+    <t>2026-10-24T08:19:36.025Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/miles-and-more</t>
@@ -7432,7 +7432,7 @@
     <t>gb/en/baggage</t>
   </si>
   <si>
-    <t>2026-10-24T00:58:54.876Z</t>
+    <t>2026-10-24T08:19:38.430Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/baggage</t>
@@ -8032,7 +8032,7 @@
     <t>gb/en/flight-search</t>
   </si>
   <si>
-    <t>2026-10-24T00:56:16.733Z</t>
+    <t>2026-10-24T08:28:20.153Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/flight-search</t>
@@ -8176,7 +8176,7 @@
     <t>gb/en/general-conditions-currency-conversion</t>
   </si>
   <si>
-    <t>2026-10-23T05:23:15.158Z</t>
+    <t>2026-10-24T08:19:53.283Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/general-conditions-currency-conversion</t>
@@ -8584,7 +8584,7 @@
     <t>gb/en/miles-and-more</t>
   </si>
   <si>
-    <t>2026-10-24T00:59:06.791Z</t>
+    <t>2026-10-24T08:19:40.985Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/miles-and-more</t>
@@ -8968,7 +8968,7 @@
     <t>gb/en/sepa-terms-and-conditions-b</t>
   </si>
   <si>
-    <t>2026-10-23T05:24:09.032Z</t>
+    <t>2026-10-24T08:19:55.410Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/sepa-terms-and-conditions-b</t>
@@ -9100,7 +9100,7 @@
     <t>gb/en/terms-and-conditions-lh</t>
   </si>
   <si>
-    <t>2026-10-23T05:24:20.354Z</t>
+    <t>2026-10-24T08:19:58.361Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/terms-and-conditions-lh</t>
@@ -10837,7 +10837,7 @@
     <t>gb/en/common/accessibility-statement</t>
   </si>
   <si>
-    <t>2026-10-23T05:13:55.116Z</t>
+    <t>2026-10-24T08:19:51.399Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/common/accessibility-statement</t>

</xml_diff>